<commit_message>
bio prices and 2050 bld rate
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan10/SuppXLS/Scen_Base_VS.xlsx
+++ b/VerveStacks_IND_grids_kan10/SuppXLS/Scen_Base_VS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan10\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD8A1FAE-5DBB-4C7F-B7AA-9D175143C8B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B977231-5413-41A7-AB0E-DFFA76CF23E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2926,9 +2926,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -3056,7 +3057,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3074,6 +3075,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Heading 3" xfId="2" builtinId="18"/>
@@ -11739,12 +11741,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B18" s="9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:10" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A19" s="8" t="s">
         <v>43</v>
       </c>
@@ -11770,10 +11772,13 @@
         <v>2040</v>
       </c>
       <c r="I19" s="8">
+        <v>2050</v>
+      </c>
+      <c r="J19" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -11799,11 +11804,15 @@
         <f>D11</f>
         <v>150</v>
       </c>
-      <c r="I20">
+      <c r="I20" s="15">
+        <f>H20*1.25</f>
+        <v>187.5</v>
+      </c>
+      <c r="J20">
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -11829,11 +11838,15 @@
         <f>F11</f>
         <v>60</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="15">
+        <f t="shared" ref="I21:I27" si="1">H21*1.25</f>
+        <v>75</v>
+      </c>
+      <c r="J21">
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>6</v>
       </c>
@@ -11842,7 +11855,7 @@
         <v>uce_buildrate_hydro</v>
       </c>
       <c r="C22" t="str">
-        <f t="shared" ref="C22:C27" si="1">A22</f>
+        <f t="shared" ref="C22:C27" si="2">A22</f>
         <v>hydro</v>
       </c>
       <c r="D22" t="s">
@@ -11862,11 +11875,15 @@
         <f>H11</f>
         <v>6</v>
       </c>
-      <c r="I22">
+      <c r="I22" s="15">
+        <f t="shared" si="1"/>
+        <v>7.5</v>
+      </c>
+      <c r="J22">
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>19</v>
       </c>
@@ -11875,7 +11892,7 @@
         <v>uce_buildrate_nuclear</v>
       </c>
       <c r="C23" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>nuclear</v>
       </c>
       <c r="D23" t="s">
@@ -11895,11 +11912,15 @@
         <f>J11</f>
         <v>6</v>
       </c>
-      <c r="I23">
+      <c r="I23" s="15">
+        <f t="shared" si="1"/>
+        <v>7.5</v>
+      </c>
+      <c r="J23">
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>924</v>
       </c>
@@ -11908,7 +11929,7 @@
         <v>uce_buildrate_geothermal</v>
       </c>
       <c r="C24" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>geothermal</v>
       </c>
       <c r="D24" t="s">
@@ -11926,11 +11947,15 @@
       <c r="H24">
         <v>0</v>
       </c>
-      <c r="I24">
+      <c r="I24" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J24">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>5</v>
       </c>
@@ -11939,7 +11964,7 @@
         <v>uce_buildrate_coal</v>
       </c>
       <c r="C25" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>coal</v>
       </c>
       <c r="D25" t="s">
@@ -11959,11 +11984,15 @@
         <f>L11</f>
         <v>31.5</v>
       </c>
-      <c r="I25">
+      <c r="I25" s="15">
+        <f t="shared" si="1"/>
+        <v>39.375</v>
+      </c>
+      <c r="J25">
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -11972,7 +12001,7 @@
         <v>uce_buildrate_gas</v>
       </c>
       <c r="C26" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>gas</v>
       </c>
       <c r="D26" t="s">
@@ -11992,11 +12021,15 @@
         <f>N11</f>
         <v>4.8000000000000007</v>
       </c>
-      <c r="I26">
+      <c r="I26" s="15">
+        <f t="shared" si="1"/>
+        <v>6.0000000000000009</v>
+      </c>
+      <c r="J26">
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>50</v>
       </c>
@@ -12005,7 +12038,7 @@
         <v>uce_buildrate_bioenergy</v>
       </c>
       <c r="C27" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>bioenergy</v>
       </c>
       <c r="D27" t="s">
@@ -12025,7 +12058,11 @@
         <f>P11</f>
         <v>15.75</v>
       </c>
-      <c r="I27">
+      <c r="I27" s="15">
+        <f t="shared" si="1"/>
+        <v>19.6875</v>
+      </c>
+      <c r="J27">
         <v>4</v>
       </c>
     </row>

</xml_diff>